<commit_message>
Add Factura C 00001-00000028 (Universidad de Palermo, julio).
Register official ARCA invoice dated 05/08/2026 for $3.250.000 as PENDIENTE in Sol monotributo billing (Excel + CSV + PDF inbox).

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/SOL/Facturacion_Monotributo_SOL_2026.xlsx
+++ b/SOL/Facturacion_Monotributo_SOL_2026.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet name="Facturación 2026" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Detalle factura 00001-00000027" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Resumen" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Detalle factura 00001-00000028" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Resumen" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,10 +20,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,8 +44,22 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -76,8 +91,23 @@
         <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D5F5E3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCF3CF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6EAF8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -99,16 +129,30 @@
         <color rgb="00B0B0B0"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -119,6 +163,20 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="3" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -487,172 +545,231 @@
   <dimension ref="A1:O7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="6" customWidth="1" min="5" max="5"/>
     <col width="6" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="55" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="50" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Facturación Monotributo — Sol 2026 (SANES MARIA SOLEDAD · CUIT 27-29039079-1)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cobro 23/07/2026 MP → destino Reserva Chris (UDESA). OpID pendiente de próximo extracto.</t>
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>Última carga: Factura C 00001-00000028 · FUNDACION UNIVERSIDAD DE PALERMO · $3.250.000 · 05/08/2026 · PENDIENTE</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>Fecha factura</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="17" t="inlineStr">
         <is>
           <t>Período desde</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="17" t="inlineStr">
         <is>
           <t>Período hasta</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="17" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="17" t="inlineStr">
         <is>
           <t>Pvta</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="17" t="inlineStr">
         <is>
           <t>Nro</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="17" t="inlineStr">
         <is>
           <t>Cliente</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" s="17" t="inlineStr">
         <is>
           <t>CUIT</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I4" s="17" t="inlineStr">
         <is>
           <t>Importe ARS</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="J4" s="17" t="inlineStr">
         <is>
           <t>CAE</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="K4" s="17" t="inlineStr">
         <is>
           <t>Vto CAE</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="L4" s="17" t="inlineStr">
         <is>
           <t>Estado cobro</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="M4" s="17" t="inlineStr">
         <is>
           <t>Fecha cobro</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="N4" s="17" t="inlineStr">
         <is>
           <t>Destino reserva</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="O4" s="17" t="inlineStr">
         <is>
           <t>PDF / comentario</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="n">
+      <c r="A5" s="18" t="n">
         <v>46226</v>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="18" t="n">
         <v>46174</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="18" t="n">
         <v>46203</v>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="19" t="inlineStr">
         <is>
           <t>FACTURA C</t>
         </is>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="E5" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="F5" s="5" t="n">
+      <c r="F5" s="19" t="n">
         <v>27</v>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G5" s="19" t="inlineStr">
         <is>
           <t>PELESSON ALDO OSCAR</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H5" s="19" t="inlineStr">
         <is>
           <t>23-14614689-9</t>
         </is>
       </c>
-      <c r="I5" s="6" t="n">
+      <c r="I5" s="20" t="n">
         <v>4900000</v>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="J5" s="19" t="inlineStr">
         <is>
           <t>86305115481677</t>
         </is>
       </c>
-      <c r="K5" s="4" t="n">
+      <c r="K5" s="18" t="n">
         <v>46236</v>
       </c>
-      <c r="L5" s="5" t="inlineStr">
+      <c r="L5" s="21" t="inlineStr">
         <is>
           <t>COBRADO</t>
         </is>
       </c>
-      <c r="M5" s="4" t="n">
+      <c r="M5" s="18" t="n">
         <v>46226</v>
       </c>
-      <c r="N5" s="5" t="inlineStr">
+      <c r="N5" s="19" t="inlineStr">
         <is>
           <t>Reserva Chris (UDESA)</t>
         </is>
       </c>
-      <c r="O5" s="5" t="inlineStr">
-        <is>
-          <t>_inbox/facturas_monotributo/27290390791_011_00001_00000027.pdf · OpID pendiente extracto</t>
+      <c r="O5" s="19" t="inlineStr">
+        <is>
+          <t>_inbox/facturas_monotributo/27290390791_011_00001_00000027.pdf · COBRADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="18" t="n">
+        <v>46239</v>
+      </c>
+      <c r="B6" s="18" t="n">
+        <v>46204</v>
+      </c>
+      <c r="C6" s="18" t="n">
+        <v>46234</v>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>FACTURA C</t>
+        </is>
+      </c>
+      <c r="E6" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="19" t="n">
+        <v>28</v>
+      </c>
+      <c r="G6" s="19" t="inlineStr">
+        <is>
+          <t>FUNDACION UNIVERSIDAD DE PALERMO</t>
+        </is>
+      </c>
+      <c r="H6" s="19" t="inlineStr">
+        <is>
+          <t>33-62010144-9</t>
+        </is>
+      </c>
+      <c r="I6" s="20" t="n">
+        <v>3250000</v>
+      </c>
+      <c r="J6" s="19" t="inlineStr">
+        <is>
+          <t>86316971456619</t>
+        </is>
+      </c>
+      <c r="K6" s="18" t="n">
+        <v>46249</v>
+      </c>
+      <c r="L6" s="22" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+      <c r="M6" s="19" t="n"/>
+      <c r="N6" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O6" s="19" t="inlineStr">
+        <is>
+          <t>_inbox/facturas_monotributo/27290390791_011_00001_00000028.pdf · PENDIENTE</t>
         </is>
       </c>
     </row>
@@ -662,20 +779,16 @@
           <t>Totales</t>
         </is>
       </c>
-      <c r="I7" s="8" t="n">
-        <v>4900000</v>
-      </c>
-      <c r="L7" s="9" t="inlineStr">
-        <is>
-          <t>1 factura · COBRADA → Reserva Chris</t>
+      <c r="I7" s="23" t="n">
+        <v>8150000</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2 facturas · 1 COBRADA(S) · 1 PENDIENTE(S)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A2:O2"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -686,22 +799,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="110" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Factura C 00001-00000027 — ARCA + cobro → Reserva Chris</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Emisor</t>
         </is>
@@ -713,7 +826,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>CUIT emisor</t>
         </is>
@@ -725,7 +838,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Tipo comprobante</t>
         </is>
@@ -737,7 +850,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Fecha de emisión</t>
         </is>
@@ -749,7 +862,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Período facturado</t>
         </is>
@@ -761,7 +874,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Cliente</t>
         </is>
@@ -773,7 +886,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>CUIT cliente</t>
         </is>
@@ -785,125 +898,194 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Domicilio cliente</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>25 De Mayo 487 Piso:2 - Capital Federal, Ciudad de Buenos Aires</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Condición IVA cliente</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>IVA Responsable Inscripto</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Honorarios profesionales por asesoramiento para la implementación de mejoras en el marco de control interno, políticas y procedimientos (Consultoría de sistemas.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>Importe Total</t>
         </is>
       </c>
-      <c r="B10" s="11" t="n">
+      <c r="B13" s="24" t="n">
         <v>4900000</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>CAE N°</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>86305115481677</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>Fecha vto. CAE</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>2026-08-02</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Vto. pago</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Condición de venta</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Otros medios de pago electrónico</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>Estado cobro</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B18" s="25" t="inlineStr">
         <is>
           <t>COBRADO</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>Fecha cobro</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>2026-07-23</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>Medio cobro</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Mercado Pago</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>Monto cobrado</t>
         </is>
       </c>
-      <c r="B16" s="11" t="n">
+      <c r="B21" t="n">
         <v>4900000</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>Destino</t>
         </is>
       </c>
-      <c r="B17" s="12" t="inlineStr">
-        <is>
-          <t>Reserva Chris (Dinero reservado Chris / UDESA)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Reserva Chris (UDESA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>OpID cobro/reserva</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>PENDIENTE próximo extracto MP (último extracto corta 2026-07-18)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
         <is>
           <t>Archivo PDF</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>_inbox/facturas_monotributo/27290390791_011_00001_00000027.pdf</t>
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Emisor SANES MARIA SOLEDAD CUIT 27-29039079-1 · Comp. 00001-00000027 · PDF ARCA · Abonada 23/07/2026 con MP · dinero a Dinero reservado Chris · OpID pendiente de próximo extracto</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -914,41 +1096,346 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>Factura C 00001-00000028 — ARCA · cobro PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Emisor</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>SANES MARIA SOLEDAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>CUIT emisor</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>27-29039079-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Tipo comprobante</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>FACTURA C (COD. 011) 00001-00000028</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Fecha de emisión</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Período facturado</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-07-01 a 2026-07-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Cliente</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>FUNDACION UNIVERSIDAD DE PALERMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>CUIT cliente</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>33-62010144-9</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Domicilio cliente</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Bravo Mario 1050 - Capital Federal, Ciudad de Buenos Aires</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Condición IVA cliente</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>IVA Sujeto Exento</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Honorarios profesionales Julio (Consultoría de sistemas.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Importe Total</t>
+        </is>
+      </c>
+      <c r="B13" s="24" t="n">
+        <v>3250000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>CAE N°</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>86316971456619</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Fecha vto. CAE</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Vto. pago</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Condición de venta</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Otros medios de pago electrónico</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Estado cobro</t>
+        </is>
+      </c>
+      <c r="B18" s="26" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Fecha cobro</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Medio cobro</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Monto cobrado</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Destino</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>— (sin ruteo a reserva)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>OpID cobro/reserva</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Archivo PDF</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>_inbox/facturas_monotributo/27290390791_011_00001_00000028.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Emisor SANES MARIA SOLEDAD CUIT 27-29039079-1 · Comp. 00001-00000028 · PDF ARCA · Cliente FUNDACION UNIVERSIDAD DE PALERMO · Período julio 2026 · Cobro PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Resumen Facturación Monotributo Sol</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="27" t="inlineStr">
         <is>
           <t>Cliente</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="27" t="inlineStr">
         <is>
           <t>CUIT</t>
         </is>
       </c>
-      <c r="C3" s="13" t="inlineStr">
+      <c r="C3" s="27" t="inlineStr">
         <is>
           <t>Comp.</t>
         </is>
       </c>
-      <c r="D3" s="13" t="inlineStr">
+      <c r="D3" s="27" t="inlineStr">
         <is>
           <t>Facturado ARS</t>
+        </is>
+      </c>
+      <c r="E3" s="27" t="inlineStr">
+        <is>
+          <t>Estado</t>
         </is>
       </c>
     </row>
@@ -968,79 +1455,115 @@
           <t>00001-00000027</t>
         </is>
       </c>
-      <c r="D4" s="11" t="n">
+      <c r="D4" s="24" t="n">
         <v>4900000</v>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="E4" s="25" t="inlineStr">
+        <is>
+          <t>COBRADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>FUNDACION UNIVERSIDAD DE PALERMO</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>33-62010144-9</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>00001-00000028</t>
+        </is>
+      </c>
+      <c r="D5" s="24" t="n">
+        <v>3250000</v>
+      </c>
+      <c r="E5" s="26" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
-      <c r="C6" s="13" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Importe ARS</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="26" t="inlineStr">
         <is>
           <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" s="11" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>COBRADO → Reserva Chris</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>1</v>
       </c>
-      <c r="C8" s="14" t="n">
+      <c r="C8" s="24" t="n">
+        <v>3250000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="25" t="inlineStr">
+        <is>
+          <t>COBRADO</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="24" t="n">
         <v>4900000</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>Total facturado</t>
         </is>
       </c>
-      <c r="C10" s="8" t="n">
-        <v>4900000</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Destino cobro</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Reserva Chris (UDESA) · Dinero reservado Chris</t>
+      <c r="C11" s="28" t="n">
+        <v>8150000</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>00001-00000027 → Reserva Chris (UDESA) · COBRADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>00001-00000028 → FUNDACION UNIVERSIDAD DE PALERMO · PENDIENTE (no es Reserva Chris)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>